<commit_message>
calculating the distribution for each feature variable
</commit_message>
<xml_diff>
--- a/source/output.xlsx
+++ b/source/output.xlsx
@@ -484,16 +484,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1924329170449599</v>
+        <v>0.19243291704496</v>
       </c>
       <c r="D3" t="n">
-        <v>6.465788564807214e-74</v>
+        <v>8.855783885743232e-26</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.006175438014218626</v>
+        <v>-0.006175438014218627</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5631228622316575</v>
+        <v>0.7385802546674562</v>
       </c>
     </row>
     <row r="4">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7357216906875989</v>
+        <v>0.7357216906875986</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8101423364901171</v>
+        <v>0.8101423364901172</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -532,16 +532,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6507208202748834</v>
+        <v>0.6507208202748833</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5764542068763481</v>
+        <v>0.5764542068763482</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1.620668679612184e-258</v>
       </c>
     </row>
     <row r="6">
@@ -559,7 +559,7 @@
         <v>0.5270006805549071</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1.196520482798497e-208</v>
       </c>
       <c r="E6" t="n">
         <v>0.678503369789944</v>
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.7561435643892088</v>
+        <v>0.7561435643892087</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8375058678828599</v>
+        <v>0.83750586788286</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.8536058035354178</v>
+        <v>0.8536058035354177</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9218749907899798</v>
+        <v>0.9218749907899799</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9234918828276372</v>
+        <v>0.9234918828276371</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.7591464722668152</v>
+        <v>0.7591464722668153</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.814008792339278</v>
+        <v>0.8140087923392779</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8570717594710896</v>
+        <v>0.8570717594710898</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5670732446468155</v>
+        <v>0.5684727299689658</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>6.88300222684879e-250</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5102688149832127</v>
+        <v>0.5099218927224485</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2.862243632667048e-193</v>
       </c>
     </row>
     <row r="13">
@@ -724,16 +724,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.3804040237552211</v>
+        <v>0.3563488844225775</v>
       </c>
       <c r="D13" t="n">
-        <v>5.959553720780655e-300</v>
+        <v>3.011554709451239e-88</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3570458973800983</v>
+        <v>0.3398151892953558</v>
       </c>
       <c r="F13" t="n">
-        <v>5.787577252416711e-262</v>
+        <v>6.417107963704902e-80</v>
       </c>
     </row>
     <row r="14">
@@ -748,16 +748,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.3408724811364616</v>
+        <v>0.313299611122669</v>
       </c>
       <c r="D14" t="n">
-        <v>1.791022551291699e-237</v>
+        <v>1.382952935969628e-67</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3482939178534328</v>
+        <v>0.3234651887045832</v>
       </c>
       <c r="F14" t="n">
-        <v>1.566161604565199e-248</v>
+        <v>3.613664906637146e-72</v>
       </c>
     </row>
     <row r="15">
@@ -772,16 +772,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.5962543989652713</v>
+        <v>0.628577020052814</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>3.231189323801752e-321</v>
       </c>
       <c r="E15" t="n">
-        <v>0.5484095268529942</v>
+        <v>0.6173697683708295</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>9.851530546739947e-307</v>
       </c>
     </row>
     <row r="16">
@@ -796,13 +796,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.4661975474024565</v>
+        <v>0.6727347821300382</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4774599582613798</v>
+        <v>0.6564237649531524</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -820,13 +820,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.4406584047088115</v>
+        <v>0.6291109304196083</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>6.422853395936205e-322</v>
       </c>
       <c r="E17" t="n">
-        <v>0.4715663975722653</v>
+        <v>0.6489019349583954</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -844,16 +844,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1924329170449599</v>
+        <v>0.19243291704496</v>
       </c>
       <c r="D18" t="n">
-        <v>6.465788564807214e-74</v>
+        <v>8.855783885743232e-26</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.006175438014218626</v>
+        <v>-0.006175438014218627</v>
       </c>
       <c r="F18" t="n">
-        <v>0.5631228622316575</v>
+        <v>0.7385802546674562</v>
       </c>
     </row>
     <row r="19">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>0.9999999999999998</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>1</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.9999999999999998</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -895,13 +895,13 @@
         <v>-0.02671460420934117</v>
       </c>
       <c r="D20" t="n">
-        <v>0.01235902762197192</v>
+        <v>0.1487505070342335</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.05611670235479525</v>
+        <v>-0.05611670235479527</v>
       </c>
       <c r="F20" t="n">
-        <v>1.453715550643508e-07</v>
+        <v>0.002405110423397167</v>
       </c>
     </row>
     <row r="21">
@@ -916,16 +916,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.2152971032970218</v>
+        <v>0.2152971032970219</v>
       </c>
       <c r="D21" t="n">
-        <v>1.747894420251479e-92</v>
+        <v>5.356203009407043e-32</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.04588858183715512</v>
+        <v>-0.04588858183715513</v>
       </c>
       <c r="F21" t="n">
-        <v>1.717303422736975e-05</v>
+        <v>0.01309402303844992</v>
       </c>
     </row>
     <row r="22">
@@ -940,16 +940,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-0.02691333248023583</v>
+        <v>-0.02691333248023584</v>
       </c>
       <c r="D22" t="n">
-        <v>0.01172412734192768</v>
+        <v>0.1457511125969876</v>
       </c>
       <c r="E22" t="n">
         <v>-0.01598210281241137</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1345251541916348</v>
+        <v>0.3877228309047636</v>
       </c>
     </row>
     <row r="23">
@@ -964,16 +964,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-0.001421995438574795</v>
+        <v>-0.001421995438574799</v>
       </c>
       <c r="D23" t="n">
-        <v>0.8940819365941522</v>
+        <v>0.9387452447027028</v>
       </c>
       <c r="E23" t="n">
-        <v>0.04352200435143277</v>
+        <v>0.04352200435143278</v>
       </c>
       <c r="F23" t="n">
-        <v>4.56442191671693e-05</v>
+        <v>0.01861682961986406</v>
       </c>
     </row>
     <row r="24">
@@ -988,16 +988,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.1970636420256235</v>
+        <v>0.1970636420256236</v>
       </c>
       <c r="D24" t="n">
-        <v>1.703363877394723e-77</v>
+        <v>5.596785946280691e-27</v>
       </c>
       <c r="E24" t="n">
         <v>-0.01542425642119473</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1486679049991231</v>
+        <v>0.4045053729971043</v>
       </c>
     </row>
     <row r="25">
@@ -1015,13 +1015,13 @@
         <v>0.03289683527731477</v>
       </c>
       <c r="D25" t="n">
-        <v>0.002063405996624037</v>
+        <v>0.07535778565979596</v>
       </c>
       <c r="E25" t="n">
-        <v>0.05507697224483302</v>
+        <v>0.05507697224483303</v>
       </c>
       <c r="F25" t="n">
-        <v>2.45960418770082e-07</v>
+        <v>0.002894631448337425</v>
       </c>
     </row>
     <row r="26">
@@ -1036,16 +1036,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.1622452866516744</v>
+        <v>0.1622452866516745</v>
       </c>
       <c r="D26" t="n">
-        <v>8.594856493811477e-53</v>
+        <v>1.079602261026082e-18</v>
       </c>
       <c r="E26" t="n">
         <v>0.08798439936918626</v>
       </c>
       <c r="F26" t="n">
-        <v>1.53238937101564e-16</v>
+        <v>1.897329145939435e-06</v>
       </c>
     </row>
     <row r="27">
@@ -1060,16 +1060,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>-0.006193425526774746</v>
+        <v>-0.006193425526774749</v>
       </c>
       <c r="D27" t="n">
-        <v>0.5619864729076206</v>
+        <v>0.7378467612699779</v>
       </c>
       <c r="E27" t="n">
         <v>0.03333228346491916</v>
       </c>
       <c r="F27" t="n">
-        <v>0.001797762338643773</v>
+        <v>0.07157179673421588</v>
       </c>
     </row>
     <row r="28">
@@ -1084,16 +1084,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.01018635663702321</v>
+        <v>0.02136207992481769</v>
       </c>
       <c r="D28" t="n">
-        <v>0.3402005177178452</v>
+        <v>0.248264997446791</v>
       </c>
       <c r="E28" t="n">
-        <v>0.002092767924329311</v>
+        <v>0.02881592477610772</v>
       </c>
       <c r="F28" t="n">
-        <v>0.8446530459048818</v>
+        <v>0.1193319946773844</v>
       </c>
     </row>
     <row r="29">
@@ -1108,16 +1108,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.03556791456214932</v>
+        <v>0.04904760331398789</v>
       </c>
       <c r="D29" t="n">
-        <v>0.000864528154016306</v>
+        <v>0.007996685747225583</v>
       </c>
       <c r="E29" t="n">
-        <v>0.02258309947248789</v>
+        <v>0.05207928064780148</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0344541599910787</v>
+        <v>0.004857097301179664</v>
       </c>
     </row>
     <row r="30">
@@ -1132,16 +1132,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.03933753877822468</v>
+        <v>0.05328252544415384</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0002290767573875307</v>
+        <v>0.003957588779356236</v>
       </c>
       <c r="E30" t="n">
-        <v>0.03107442286039943</v>
+        <v>0.05892823236329751</v>
       </c>
       <c r="F30" t="n">
-        <v>0.003612111865458417</v>
+        <v>0.001435834573158047</v>
       </c>
     </row>
     <row r="31">
@@ -1156,16 +1156,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>-0.006270023464504975</v>
+        <v>-0.02123838118700429</v>
       </c>
       <c r="D31" t="n">
-        <v>0.5571597220133419</v>
+        <v>0.2510153606089161</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.02733332888341927</v>
+        <v>-0.04200584302493247</v>
       </c>
       <c r="F31" t="n">
-        <v>0.01047666063015807</v>
+        <v>0.02314289370526412</v>
       </c>
     </row>
     <row r="32">
@@ -1180,16 +1180,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.02697172857219367</v>
+        <v>-0.0001618543403799659</v>
       </c>
       <c r="D32" t="n">
-        <v>0.01154314507902686</v>
+        <v>0.9930210918079525</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03049910076868118</v>
+        <v>0.03829958830482363</v>
       </c>
       <c r="F32" t="n">
-        <v>0.004286333051198726</v>
+        <v>0.03840249404038574</v>
       </c>
     </row>
     <row r="33">
@@ -1204,16 +1204,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.02701923365697489</v>
+        <v>0.001022159890245561</v>
       </c>
       <c r="D33" t="n">
-        <v>0.01139774940279815</v>
+        <v>0.9559478815990498</v>
       </c>
       <c r="E33" t="n">
-        <v>0.03120036263957241</v>
+        <v>0.0367581525922807</v>
       </c>
       <c r="F33" t="n">
-        <v>0.003478044224510393</v>
+        <v>0.04690657714764744</v>
       </c>
     </row>
     <row r="34">
@@ -1228,13 +1228,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.7357216906875989</v>
+        <v>0.7357216906875986</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>0.8101423364901171</v>
+        <v>0.8101423364901172</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1255,13 +1255,13 @@
         <v>-0.02671460420934117</v>
       </c>
       <c r="D35" t="n">
-        <v>0.01235902762197192</v>
+        <v>0.1487505070342335</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.05611670235479526</v>
+        <v>-0.05611670235479527</v>
       </c>
       <c r="F35" t="n">
-        <v>1.453715550643495e-07</v>
+        <v>0.002405110423397167</v>
       </c>
     </row>
     <row r="36">
@@ -1300,16 +1300,16 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.4520977501719116</v>
+        <v>0.4520977501719117</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>3.048771003674086e-147</v>
       </c>
       <c r="E37" t="n">
         <v>0.552382982617644</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>3.384440732235283e-233</v>
       </c>
     </row>
     <row r="38">
@@ -1324,10 +1324,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.4990961343555267</v>
+        <v>0.4990961343555268</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>5.764275788167167e-184</v>
       </c>
       <c r="E38" t="n">
         <v>0.6822881300127996</v>
@@ -1372,7 +1372,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.7877525039759078</v>
+        <v>0.7877525039759077</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1396,13 +1396,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.7899808396825204</v>
+        <v>0.7899808396825205</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>0.8662016713119962</v>
+        <v>0.8662016713119961</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1423,10 +1423,10 @@
         <v>0.5497467507388487</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1.507205117992564e-230</v>
       </c>
       <c r="E42" t="n">
-        <v>0.77760078228694</v>
+        <v>0.7776007822869401</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.7545405682512193</v>
+        <v>0.7545405682512194</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1468,16 +1468,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.760419829557472</v>
+        <v>0.7890124800257879</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>0.5022567308757648</v>
+        <v>0.5112367995252334</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>2.011876431627369e-194</v>
       </c>
     </row>
     <row r="45">
@@ -1492,16 +1492,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.3122521915572819</v>
+        <v>0.3127661477912633</v>
       </c>
       <c r="D45" t="n">
-        <v>1.365740522621185e-197</v>
+        <v>2.379013604190403e-67</v>
       </c>
       <c r="E45" t="n">
-        <v>0.3110540411491128</v>
+        <v>0.2978604677688969</v>
       </c>
       <c r="F45" t="n">
-        <v>5.148879785189463e-196</v>
+        <v>5.814663421907969e-61</v>
       </c>
     </row>
     <row r="46">
@@ -1516,16 +1516,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.2499247158382008</v>
+        <v>0.2476585478192828</v>
       </c>
       <c r="D46" t="n">
-        <v>5.552230875591728e-125</v>
+        <v>4.216682433567577e-42</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3000647671265144</v>
+        <v>0.2806919673166815</v>
       </c>
       <c r="F46" t="n">
-        <v>6.751879545148911e-182</v>
+        <v>4.638489294353465e-54</v>
       </c>
     </row>
     <row r="47">
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.8162022175137895</v>
+        <v>0.8874025204297278</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>0.6666910856063926</v>
+        <v>0.7725366917449679</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1564,13 +1564,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.3984232096795318</v>
+        <v>0.6017818671719291</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1.54678419033053e-287</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4831313822728238</v>
+        <v>0.68003028541919</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -1588,13 +1588,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.3570432489558609</v>
+        <v>0.5326142466146806</v>
       </c>
       <c r="D49" t="n">
-        <v>5.842872470064653e-262</v>
+        <v>6.730756418763045e-214</v>
       </c>
       <c r="E49" t="n">
-        <v>0.4799749441437264</v>
+        <v>0.6784089636963448</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1621,7 +1621,7 @@
         <v>0.5764542068763482</v>
       </c>
       <c r="F50" t="n">
-        <v>0</v>
+        <v>1.620668679612184e-258</v>
       </c>
     </row>
     <row r="51">
@@ -1636,16 +1636,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.2152971032970218</v>
+        <v>0.2152971032970219</v>
       </c>
       <c r="D51" t="n">
-        <v>1.747894420251479e-92</v>
+        <v>5.356203009407043e-32</v>
       </c>
       <c r="E51" t="n">
-        <v>-0.04588858183715512</v>
+        <v>-0.04588858183715513</v>
       </c>
       <c r="F51" t="n">
-        <v>1.717303422736975e-05</v>
+        <v>0.0130940230384499</v>
       </c>
     </row>
     <row r="52">
@@ -1660,16 +1660,16 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.4520977501719116</v>
+        <v>0.4520977501719117</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>3.048771003674086e-147</v>
       </c>
       <c r="E52" t="n">
-        <v>0.552382982617644</v>
+        <v>0.5523829826176441</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>3.384440732233742e-233</v>
       </c>
     </row>
     <row r="53">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.5287915178516048</v>
+        <v>0.5287915178516049</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>2.593240488385913e-210</v>
       </c>
       <c r="E54" t="n">
         <v>0.5856303844701728</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>9.799917396078863e-269</v>
       </c>
     </row>
     <row r="55">
@@ -1732,16 +1732,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.6325317173487343</v>
+        <v>0.6325317173487341</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0.593000069121981</v>
+        <v>0.5930000691219809</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>3.503514259446345e-277</v>
       </c>
     </row>
     <row r="56">
@@ -1759,13 +1759,13 @@
         <v>0.5576761593767621</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>1.377576267002501e-238</v>
       </c>
       <c r="E56" t="n">
         <v>0.5229865546594921</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>5.913344801983622e-205</v>
       </c>
     </row>
     <row r="57">
@@ -1783,13 +1783,13 @@
         <v>0.5723084535866328</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>5.25924660959426e-254</v>
       </c>
       <c r="E57" t="n">
-        <v>0.5430243412783181</v>
+        <v>0.5430243412783182</v>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>6.702385417670291e-224</v>
       </c>
     </row>
     <row r="58">
@@ -1807,13 +1807,13 @@
         <v>0.5301995041044169</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1.254526768946847e-211</v>
       </c>
       <c r="E58" t="n">
-        <v>0.4627060350439275</v>
+        <v>0.4627060350439274</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>4.894808930882772e-155</v>
       </c>
     </row>
     <row r="59">
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.648218207719039</v>
+        <v>0.6482182077190393</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1837,7 +1837,7 @@
         <v>0.6103058781014912</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>6.686767738481168e-298</v>
       </c>
     </row>
     <row r="60">
@@ -1852,16 +1852,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.3216738536245097</v>
+        <v>0.3377286666969999</v>
       </c>
       <c r="D60" t="n">
-        <v>3.033455259270989e-210</v>
+        <v>6.651981994021564e-79</v>
       </c>
       <c r="E60" t="n">
-        <v>0.3742853801281313</v>
+        <v>0.3727386080762574</v>
       </c>
       <c r="F60" t="n">
-        <v>1.078262449473593e-289</v>
+        <v>5.217798937917992e-97</v>
       </c>
     </row>
     <row r="61">
@@ -1876,16 +1876,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.3072852859526205</v>
+        <v>0.3051606447703192</v>
       </c>
       <c r="D61" t="n">
-        <v>4.190682509214775e-191</v>
+        <v>4.81482132939331e-64</v>
       </c>
       <c r="E61" t="n">
-        <v>0.2734766478441396</v>
+        <v>0.2677579467456537</v>
       </c>
       <c r="F61" t="n">
-        <v>3.22464742660719e-150</v>
+        <v>3.566234961241895e-49</v>
       </c>
     </row>
     <row r="62">
@@ -1900,16 +1900,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.2709268150383519</v>
+        <v>0.2669209206728209</v>
       </c>
       <c r="D62" t="n">
-        <v>2.326242065173933e-147</v>
+        <v>7.232289635408424e-49</v>
       </c>
       <c r="E62" t="n">
-        <v>0.2489887219065404</v>
+        <v>0.2417839643056925</v>
       </c>
       <c r="F62" t="n">
-        <v>4.944103699853044e-124</v>
+        <v>3.760334409000857e-40</v>
       </c>
     </row>
     <row r="63">
@@ -1924,16 +1924,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.3301780681499282</v>
+        <v>0.3290533978379733</v>
       </c>
       <c r="D63" t="n">
-        <v>4.599953061782032e-222</v>
+        <v>9.165099730651372e-75</v>
       </c>
       <c r="E63" t="n">
-        <v>0.373118984834427</v>
+        <v>0.4105381974221958</v>
       </c>
       <c r="F63" t="n">
-        <v>9.185084275076665e-288</v>
+        <v>3.034812928967799e-119</v>
       </c>
     </row>
     <row r="64">
@@ -1948,16 +1948,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.3715616261543613</v>
+        <v>0.4985624511795598</v>
       </c>
       <c r="D64" t="n">
-        <v>3.373432845809345e-285</v>
+        <v>1.624781270499516e-183</v>
       </c>
       <c r="E64" t="n">
-        <v>0.3532439313403115</v>
+        <v>0.4682609954027203</v>
       </c>
       <c r="F64" t="n">
-        <v>4.468890820878274e-256</v>
+        <v>3.140302652040833e-159</v>
       </c>
     </row>
     <row r="65">
@@ -1972,16 +1972,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.3698856612386199</v>
+        <v>0.4991921632127196</v>
       </c>
       <c r="D65" t="n">
-        <v>1.873329941423436e-282</v>
+        <v>4.782771346255567e-184</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3471667045967565</v>
+        <v>0.4635132422849853</v>
       </c>
       <c r="F65" t="n">
-        <v>7.832752125756156e-247</v>
+        <v>1.216968915903044e-155</v>
       </c>
     </row>
     <row r="66">
@@ -1999,7 +1999,7 @@
         <v>0.5270006805549071</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1.196520482798497e-208</v>
       </c>
       <c r="E66" t="n">
         <v>0.6785033697899441</v>
@@ -2020,16 +2020,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.02691333248023583</v>
+        <v>-0.02691333248023584</v>
       </c>
       <c r="D67" t="n">
-        <v>0.01172412734192768</v>
+        <v>0.1457511125969876</v>
       </c>
       <c r="E67" t="n">
         <v>-0.01598210281241137</v>
       </c>
       <c r="F67" t="n">
-        <v>0.1345251541916348</v>
+        <v>0.3877228309047636</v>
       </c>
     </row>
     <row r="68">
@@ -2044,13 +2044,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.4990961343555267</v>
+        <v>0.4990961343555268</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>5.764275788167167e-184</v>
       </c>
       <c r="E68" t="n">
-        <v>0.6822881300127996</v>
+        <v>0.6822881300127998</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -2068,16 +2068,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.5287915178516047</v>
+        <v>0.5287915178516049</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>2.593240488385913e-210</v>
       </c>
       <c r="E69" t="n">
-        <v>0.5856303844701728</v>
+        <v>0.5856303844701727</v>
       </c>
       <c r="F69" t="n">
-        <v>0</v>
+        <v>9.799917396083321e-269</v>
       </c>
     </row>
     <row r="70">
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
         <v>0.9999999999999999</v>
-      </c>
-      <c r="D70" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" t="n">
-        <v>0.9999999999999998</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -2119,7 +2119,7 @@
         <v>0.6079231516744814</v>
       </c>
       <c r="D71" t="n">
-        <v>0</v>
+        <v>5.677073252013767e-295</v>
       </c>
       <c r="E71" t="n">
         <v>0.6761616831230379</v>
@@ -2143,13 +2143,13 @@
         <v>0.4471944519874925</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>9.875284630260631e-144</v>
       </c>
       <c r="E72" t="n">
         <v>0.5775515581247451</v>
       </c>
       <c r="F72" t="n">
-        <v>0</v>
+        <v>1.010996146213671e-259</v>
       </c>
     </row>
     <row r="73">
@@ -2164,10 +2164,10 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.5993442827736034</v>
+        <v>0.5993442827736035</v>
       </c>
       <c r="D73" t="n">
-        <v>0</v>
+        <v>1.247327012565619e-284</v>
       </c>
       <c r="E73" t="n">
         <v>0.7326915001787035</v>
@@ -2188,10 +2188,10 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.607856223035797</v>
+        <v>0.6078562230357971</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>6.855439674183524e-295</v>
       </c>
       <c r="E74" t="n">
         <v>0.6748645126014037</v>
@@ -2212,13 +2212,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.5724544220071908</v>
+        <v>0.5724544220071909</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>3.657467494590659e-254</v>
       </c>
       <c r="E75" t="n">
-        <v>0.6755834327850319</v>
+        <v>0.6755834327850316</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -2236,16 +2236,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.3898379176770721</v>
+        <v>0.4035643370018586</v>
       </c>
       <c r="D76" t="n">
-        <v>3.325232842038179e-316</v>
+        <v>6.396129474769507e-115</v>
       </c>
       <c r="E76" t="n">
-        <v>0.4110417597634477</v>
+        <v>0.4141971159420432</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
+        <v>1.486165612633583e-121</v>
       </c>
     </row>
     <row r="77">
@@ -2260,16 +2260,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.2790712506792598</v>
+        <v>0.2847902877252663</v>
       </c>
       <c r="D77" t="n">
-        <v>1.343933497167525e-156</v>
+        <v>1.154579806920999e-55</v>
       </c>
       <c r="E77" t="n">
-        <v>0.2632974146446778</v>
+        <v>0.2592221647068217</v>
       </c>
       <c r="F77" t="n">
-        <v>5.42694288762349e-139</v>
+        <v>4.287620295322336e-46</v>
       </c>
     </row>
     <row r="78">
@@ -2284,16 +2284,16 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.2768588934974741</v>
+        <v>0.2746780170093809</v>
       </c>
       <c r="D78" t="n">
-        <v>4.669965564166831e-154</v>
+        <v>9.358965268045693e-52</v>
       </c>
       <c r="E78" t="n">
-        <v>0.2607033179582323</v>
+        <v>0.2515153802441716</v>
       </c>
       <c r="F78" t="n">
-        <v>3.291013377008714e-136</v>
+        <v>2.070398809270135e-43</v>
       </c>
     </row>
     <row r="79">
@@ -2308,16 +2308,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.3703949996998294</v>
+        <v>0.3965453382286718</v>
       </c>
       <c r="D79" t="n">
-        <v>2.755846669117891e-283</v>
+        <v>1.133556306195914e-110</v>
       </c>
       <c r="E79" t="n">
-        <v>0.4374669261133945</v>
+        <v>0.5018445951260091</v>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>2.693349665732633e-186</v>
       </c>
     </row>
     <row r="80">
@@ -2332,16 +2332,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.3089852309067529</v>
+        <v>0.4561969243634081</v>
       </c>
       <c r="D80" t="n">
-        <v>2.607758478347649e-193</v>
+        <v>3.198415177047571e-150</v>
       </c>
       <c r="E80" t="n">
-        <v>0.3582279529335334</v>
+        <v>0.501312573825911</v>
       </c>
       <c r="F80" t="n">
-        <v>8.230089132646972e-264</v>
+        <v>7.639505610511546e-186</v>
       </c>
     </row>
     <row r="81">
@@ -2356,16 +2356,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.3302646504115752</v>
+        <v>0.4874773034984594</v>
       </c>
       <c r="D81" t="n">
-        <v>3.471009545346545e-222</v>
+        <v>2.401189319370942e-174</v>
       </c>
       <c r="E81" t="n">
-        <v>0.3602639731468211</v>
+        <v>0.5044367858557851</v>
       </c>
       <c r="F81" t="n">
-        <v>5.192471947474459e-267</v>
+        <v>1.631999756783036e-188</v>
       </c>
     </row>
     <row r="82">
@@ -2380,13 +2380,13 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.7561435643892088</v>
+        <v>0.7561435643892087</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
       </c>
       <c r="E82" t="n">
-        <v>0.8375058678828599</v>
+        <v>0.83750586788286</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2404,16 +2404,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-0.001421995438574794</v>
+        <v>-0.001421995438574796</v>
       </c>
       <c r="D83" t="n">
-        <v>0.8940819365941522</v>
+        <v>0.9387452447027028</v>
       </c>
       <c r="E83" t="n">
-        <v>0.04352200435143277</v>
+        <v>0.04352200435143278</v>
       </c>
       <c r="F83" t="n">
-        <v>4.56442191671693e-05</v>
+        <v>0.01861682961986406</v>
       </c>
     </row>
     <row r="84">
@@ -2452,7 +2452,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.6325317173487343</v>
+        <v>0.6325317173487341</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -2461,7 +2461,7 @@
         <v>0.593000069121981</v>
       </c>
       <c r="F85" t="n">
-        <v>0</v>
+        <v>3.503514259445547e-277</v>
       </c>
     </row>
     <row r="86">
@@ -2479,7 +2479,7 @@
         <v>0.6079231516744814</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>5.677073252013767e-295</v>
       </c>
       <c r="E86" t="n">
         <v>0.6761616831230379</v>
@@ -2506,7 +2506,7 @@
         <v>0</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
       <c r="E88" t="n">
-        <v>0.7510544655741759</v>
+        <v>0.7510544655741758</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -2548,13 +2548,13 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.8436219495427355</v>
+        <v>0.8436219495427356</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
       </c>
       <c r="E89" t="n">
-        <v>0.9061590804702223</v>
+        <v>0.9061590804702222</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.8078116381495783</v>
+        <v>0.8078116381495786</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -2596,13 +2596,13 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0.9560728157110109</v>
+        <v>0.956072815711011</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>0.9879795733556364</v>
+        <v>0.9879795733556361</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2620,16 +2620,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.4682599022735286</v>
+        <v>0.4775889959796604</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>1.904024295814503e-166</v>
       </c>
       <c r="E92" t="n">
-        <v>0.5151193076879514</v>
+        <v>0.5309792149274541</v>
       </c>
       <c r="F92" t="n">
-        <v>0</v>
+        <v>2.330146312206435e-212</v>
       </c>
     </row>
     <row r="93">
@@ -2644,16 +2644,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.4075747514081423</v>
+        <v>0.4097093086883555</v>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>1.003364342699521e-118</v>
       </c>
       <c r="E93" t="n">
-        <v>0.3653004039185452</v>
+        <v>0.3678999806840161</v>
       </c>
       <c r="F93" t="n">
-        <v>4.991471081811902e-275</v>
+        <v>2.277707968055732e-94</v>
       </c>
     </row>
     <row r="94">
@@ -2668,16 +2668,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>0.4024488583609285</v>
+        <v>0.396583011286486</v>
       </c>
       <c r="D94" t="n">
-        <v>0</v>
+        <v>1.076249882176215e-110</v>
       </c>
       <c r="E94" t="n">
-        <v>0.3632729494628876</v>
+        <v>0.3595090892907859</v>
       </c>
       <c r="F94" t="n">
-        <v>8.770362586651322e-272</v>
+        <v>6.748477013271474e-90</v>
       </c>
     </row>
     <row r="95">
@@ -2692,13 +2692,13 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>0.5019743068575309</v>
+        <v>0.5194246389965358</v>
       </c>
       <c r="D95" t="n">
-        <v>0</v>
+        <v>1.019307778738693e-201</v>
       </c>
       <c r="E95" t="n">
-        <v>0.5916864228596775</v>
+        <v>0.6748576249077125</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -2716,13 +2716,13 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.5299363870485871</v>
+        <v>0.7561706466631242</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
       </c>
       <c r="E96" t="n">
-        <v>0.5411708015366777</v>
+        <v>0.7551411147977549</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -2740,13 +2740,13 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>0.5523042907844735</v>
+        <v>0.7953303508166576</v>
       </c>
       <c r="D97" t="n">
         <v>0</v>
       </c>
       <c r="E97" t="n">
-        <v>0.5445199998267021</v>
+        <v>0.7603448776971423</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -2764,13 +2764,13 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.8536058035354178</v>
+        <v>0.8536058035354177</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8466424007951175</v>
+        <v>0.8466424007951174</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -2788,16 +2788,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.1970636420256235</v>
+        <v>0.1970636420256236</v>
       </c>
       <c r="D99" t="n">
-        <v>1.703363877394723e-77</v>
+        <v>5.596785946280691e-27</v>
       </c>
       <c r="E99" t="n">
         <v>-0.01542425642119473</v>
       </c>
       <c r="F99" t="n">
-        <v>0.1486679049991231</v>
+        <v>0.4045053729971043</v>
       </c>
     </row>
     <row r="100">
@@ -2818,7 +2818,7 @@
         <v>0</v>
       </c>
       <c r="E100" t="n">
-        <v>0.7529821190256042</v>
+        <v>0.7529821190256041</v>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -2839,13 +2839,13 @@
         <v>0.5576761593767621</v>
       </c>
       <c r="D101" t="n">
-        <v>0</v>
+        <v>1.377576267002501e-238</v>
       </c>
       <c r="E101" t="n">
         <v>0.5229865546594921</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>5.913344801983622e-205</v>
       </c>
     </row>
     <row r="102">
@@ -2863,13 +2863,13 @@
         <v>0.4471944519874925</v>
       </c>
       <c r="D102" t="n">
-        <v>0</v>
+        <v>9.875284630260631e-144</v>
       </c>
       <c r="E102" t="n">
         <v>0.5775515581247451</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>1.010996146213671e-259</v>
       </c>
     </row>
     <row r="103">
@@ -2890,7 +2890,7 @@
         <v>0</v>
       </c>
       <c r="E103" t="n">
-        <v>0.7510544655741758</v>
+        <v>0.7510544655741757</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -2932,13 +2932,13 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>0.7845496940809744</v>
+        <v>0.7845496940809745</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
       </c>
       <c r="E105" t="n">
-        <v>0.7799867853721003</v>
+        <v>0.7799867853721002</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -2956,13 +2956,13 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>0.624042958343595</v>
+        <v>0.6240429583435951</v>
       </c>
       <c r="D106" t="n">
-        <v>0</v>
+        <v>2.758880659061471e-315</v>
       </c>
       <c r="E106" t="n">
-        <v>0.7198322886308766</v>
+        <v>0.7198322886308767</v>
       </c>
       <c r="F106" t="n">
         <v>0</v>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
       <c r="E107" t="n">
-        <v>0.7648115466624597</v>
+        <v>0.7648115466624595</v>
       </c>
       <c r="F107" t="n">
         <v>0</v>
@@ -3004,16 +3004,16 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>0.6397064258770416</v>
+        <v>0.6414291219845514</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
       </c>
       <c r="E108" t="n">
-        <v>0.4996094804981535</v>
+        <v>0.486740055226751</v>
       </c>
       <c r="F108" t="n">
-        <v>0</v>
+        <v>9.514259742322854e-174</v>
       </c>
     </row>
     <row r="109">
@@ -3028,16 +3028,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>0.3363603250452208</v>
+        <v>0.3207630264187031</v>
       </c>
       <c r="D109" t="n">
-        <v>6.756398178713562e-231</v>
+        <v>6.216881795166131e-71</v>
       </c>
       <c r="E109" t="n">
-        <v>0.3303190646088017</v>
+        <v>0.3069814252586165</v>
       </c>
       <c r="F109" t="n">
-        <v>2.907871889481469e-222</v>
+        <v>7.942911745145299e-65</v>
       </c>
     </row>
     <row r="110">
@@ -3052,16 +3052,16 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>0.2977541246723888</v>
+        <v>0.2782355284792996</v>
       </c>
       <c r="D110" t="n">
-        <v>5.254068579704514e-179</v>
+        <v>4.119046442912065e-53</v>
       </c>
       <c r="E110" t="n">
-        <v>0.3270831565247423</v>
+        <v>0.2962339110355097</v>
       </c>
       <c r="F110" t="n">
-        <v>1.019080151527884e-217</v>
+        <v>2.748727289608711e-60</v>
       </c>
     </row>
     <row r="111">
@@ -3076,16 +3076,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>0.6683247652977408</v>
+        <v>0.6935080803768685</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
       </c>
       <c r="E111" t="n">
-        <v>0.5188769338767233</v>
+        <v>0.5635413535925445</v>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1.125979450288559e-244</v>
       </c>
     </row>
     <row r="112">
@@ -3100,16 +3100,16 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>0.4201886578392034</v>
+        <v>0.5685183567514941</v>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>6.153545989357209e-250</v>
       </c>
       <c r="E112" t="n">
-        <v>0.4372618026972731</v>
+        <v>0.5846701978281483</v>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>1.190708871335717e-267</v>
       </c>
     </row>
     <row r="113">
@@ -3124,16 +3124,16 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>0.3946052730366</v>
+        <v>0.5261332267278964</v>
       </c>
       <c r="D113" t="n">
-        <v>0</v>
+        <v>7.592567275135141e-208</v>
       </c>
       <c r="E113" t="n">
-        <v>0.4353205574189013</v>
+        <v>0.5820603351510775</v>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>1.012817295614129e-264</v>
       </c>
     </row>
     <row r="114">
@@ -3148,13 +3148,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0.9218749907899798</v>
+        <v>0.9218749907899799</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
       </c>
       <c r="E114" t="n">
-        <v>0.9234918828276371</v>
+        <v>0.9234918828276373</v>
       </c>
       <c r="F114" t="n">
         <v>0</v>
@@ -3172,16 +3172,16 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>0.03289683527731476</v>
+        <v>0.03289683527731477</v>
       </c>
       <c r="D115" t="n">
-        <v>0.002063405996624037</v>
+        <v>0.07535778565979596</v>
       </c>
       <c r="E115" t="n">
-        <v>0.05507697224483302</v>
+        <v>0.05507697224483303</v>
       </c>
       <c r="F115" t="n">
-        <v>2.45960418770082e-07</v>
+        <v>0.002894631448337425</v>
       </c>
     </row>
     <row r="116">
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>0.7899808396825202</v>
+        <v>0.7899808396825205</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -3223,13 +3223,13 @@
         <v>0.5723084535866328</v>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>5.25924660959426e-254</v>
       </c>
       <c r="E117" t="n">
         <v>0.5430243412783182</v>
       </c>
       <c r="F117" t="n">
-        <v>0</v>
+        <v>6.702385417670291e-224</v>
       </c>
     </row>
     <row r="118">
@@ -3244,10 +3244,10 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>0.5993442827736034</v>
+        <v>0.5993442827736035</v>
       </c>
       <c r="D118" t="n">
-        <v>0</v>
+        <v>1.247327012565619e-284</v>
       </c>
       <c r="E118" t="n">
         <v>0.7326915001787037</v>
@@ -3268,13 +3268,13 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>0.8436219495427355</v>
+        <v>0.8436219495427356</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0.9061590804702222</v>
+        <v>0.9061590804702221</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3298,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="E120" t="n">
-        <v>0.7799867853721003</v>
+        <v>0.7799867853721002</v>
       </c>
       <c r="F120" t="n">
         <v>0</v>
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>0.9999999999999997</v>
+        <v>1</v>
       </c>
       <c r="D121" t="n">
         <v>0</v>
@@ -3340,13 +3340,13 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>0.8034183001519282</v>
+        <v>0.8034183001519284</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
       </c>
       <c r="E122" t="n">
-        <v>0.9073978015773614</v>
+        <v>0.9073978015773613</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -3364,7 +3364,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>0.8954789419953444</v>
+        <v>0.8954789419953446</v>
       </c>
       <c r="D123" t="n">
         <v>0</v>
@@ -3388,16 +3388,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>0.5926228087235358</v>
+        <v>0.5954241994209174</v>
       </c>
       <c r="D124" t="n">
-        <v>0</v>
+        <v>5.224581382714567e-280</v>
       </c>
       <c r="E124" t="n">
-        <v>0.5057841390057547</v>
+        <v>0.5070053234883386</v>
       </c>
       <c r="F124" t="n">
-        <v>0</v>
+        <v>9.917867204668648e-191</v>
       </c>
     </row>
     <row r="125">
@@ -3412,16 +3412,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>0.3937841663624979</v>
+        <v>0.3803380055735273</v>
       </c>
       <c r="D125" t="n">
-        <v>3.952525166729972e-323</v>
+        <v>3.013079602062415e-101</v>
       </c>
       <c r="E125" t="n">
-        <v>0.3527963077087694</v>
+        <v>0.3402221413844022</v>
       </c>
       <c r="F125" t="n">
-        <v>2.178008683112619e-255</v>
+        <v>4.058274053945986e-80</v>
       </c>
     </row>
     <row r="126">
@@ -3436,16 +3436,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>0.3565116123064391</v>
+        <v>0.3386504491435319</v>
       </c>
       <c r="D126" t="n">
-        <v>3.933607204706318e-261</v>
+        <v>2.372692861003124e-79</v>
       </c>
       <c r="E126" t="n">
-        <v>0.3453077374009511</v>
+        <v>0.3267396849040175</v>
       </c>
       <c r="F126" t="n">
-        <v>4.793936916330531e-244</v>
+        <v>1.105450914403047e-73</v>
       </c>
     </row>
     <row r="127">
@@ -3460,13 +3460,13 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.630015091868017</v>
+        <v>0.6679093753194176</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
       </c>
       <c r="E127" t="n">
-        <v>0.5796138633438634</v>
+        <v>0.6590162017447879</v>
       </c>
       <c r="F127" t="n">
         <v>0</v>
@@ -3484,13 +3484,13 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>0.5025739628471854</v>
+        <v>0.7336547611954214</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
       </c>
       <c r="E128" t="n">
-        <v>0.5063145748881588</v>
+        <v>0.7036176710225318</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
@@ -3508,13 +3508,13 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>0.4780327375826023</v>
+        <v>0.6937593939631954</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
       </c>
       <c r="E129" t="n">
-        <v>0.4998976758143783</v>
+        <v>0.6956324365644663</v>
       </c>
       <c r="F129" t="n">
         <v>0</v>
@@ -3532,13 +3532,13 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>0.7591464722668152</v>
+        <v>0.7591464722668153</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
       </c>
       <c r="E130" t="n">
-        <v>0.8535040680934154</v>
+        <v>0.8535040680934152</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -3559,13 +3559,13 @@
         <v>0.1622452866516745</v>
       </c>
       <c r="D131" t="n">
-        <v>8.594856493811477e-53</v>
+        <v>1.079602261026082e-18</v>
       </c>
       <c r="E131" t="n">
         <v>0.08798439936918626</v>
       </c>
       <c r="F131" t="n">
-        <v>1.53238937101564e-16</v>
+        <v>1.897329145939435e-06</v>
       </c>
     </row>
     <row r="132">
@@ -3583,7 +3583,7 @@
         <v>0.5497467507388487</v>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>1.507205117992564e-230</v>
       </c>
       <c r="E132" t="n">
         <v>0.7776007822869401</v>
@@ -3607,13 +3607,13 @@
         <v>0.5301995041044167</v>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
+        <v>1.25452676894713e-211</v>
       </c>
       <c r="E133" t="n">
-        <v>0.4627060350439275</v>
+        <v>0.4627060350439274</v>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>4.894808930882772e-155</v>
       </c>
     </row>
     <row r="134">
@@ -3628,10 +3628,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>0.607856223035797</v>
+        <v>0.6078562230357971</v>
       </c>
       <c r="D134" t="n">
-        <v>0</v>
+        <v>6.855439674183524e-295</v>
       </c>
       <c r="E134" t="n">
         <v>0.6748645126014037</v>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>0.8078116381495783</v>
+        <v>0.8078116381495786</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -3676,10 +3676,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>0.624042958343595</v>
+        <v>0.6240429583435951</v>
       </c>
       <c r="D136" t="n">
-        <v>0</v>
+        <v>2.758880659061471e-315</v>
       </c>
       <c r="E136" t="n">
         <v>0.7198322886308766</v>
@@ -3700,7 +3700,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.8034183001519282</v>
+        <v>0.8034183001519284</v>
       </c>
       <c r="D137" t="n">
         <v>0</v>
@@ -3724,7 +3724,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>0.9999999999999998</v>
+        <v>1</v>
       </c>
       <c r="D138" t="n">
         <v>0</v>
@@ -3748,13 +3748,13 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>0.7437421256360544</v>
+        <v>0.7437421256360546</v>
       </c>
       <c r="D139" t="n">
         <v>0</v>
       </c>
       <c r="E139" t="n">
-        <v>0.8193256353355838</v>
+        <v>0.8193256353355837</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3772,16 +3772,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>0.4087122424828522</v>
+        <v>0.4153143148941014</v>
       </c>
       <c r="D140" t="n">
-        <v>0</v>
+        <v>2.890441153326847e-122</v>
       </c>
       <c r="E140" t="n">
-        <v>0.4582765507040158</v>
+        <v>0.4682918695866836</v>
       </c>
       <c r="F140" t="n">
-        <v>0</v>
+        <v>2.974753368755851e-159</v>
       </c>
     </row>
     <row r="141">
@@ -3796,16 +3796,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>0.3503533015298208</v>
+        <v>0.3575538183550458</v>
       </c>
       <c r="D141" t="n">
-        <v>1.181761123760613e-251</v>
+        <v>7.112860809889674e-89</v>
       </c>
       <c r="E141" t="n">
-        <v>0.320934890156163</v>
+        <v>0.3191854015970586</v>
       </c>
       <c r="F141" t="n">
-        <v>3.097555130847909e-209</v>
+        <v>3.229370326874344e-70</v>
       </c>
     </row>
     <row r="142">
@@ -3820,16 +3820,16 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>0.3691561116430948</v>
+        <v>0.3623410734346687</v>
       </c>
       <c r="D142" t="n">
-        <v>2.898801059733938e-281</v>
+        <v>2.162462502322069e-91</v>
       </c>
       <c r="E142" t="n">
-        <v>0.3282896131279908</v>
+        <v>0.3190909052808025</v>
       </c>
       <c r="F142" t="n">
-        <v>2.090738171857424e-219</v>
+        <v>3.563204494876834e-70</v>
       </c>
     </row>
     <row r="143">
@@ -3844,16 +3844,16 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>0.4233697610687855</v>
+        <v>0.4357215233182617</v>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>9.695603760244763e-136</v>
       </c>
       <c r="E143" t="n">
-        <v>0.5234867060019465</v>
+        <v>0.5955793106741324</v>
       </c>
       <c r="F143" t="n">
-        <v>0</v>
+        <v>3.438548842950038e-280</v>
       </c>
     </row>
     <row r="144">
@@ -3868,16 +3868,16 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>0.4227601785774302</v>
+        <v>0.5972439902745043</v>
       </c>
       <c r="D144" t="n">
-        <v>0</v>
+        <v>3.804793221767193e-282</v>
       </c>
       <c r="E144" t="n">
-        <v>0.4525712442293984</v>
+        <v>0.6305744038468284</v>
       </c>
       <c r="F144" t="n">
-        <v>0</v>
+        <v>9.881312916824931e-324</v>
       </c>
     </row>
     <row r="145">
@@ -3892,13 +3892,13 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>0.45402368917089</v>
+        <v>0.6490046574017936</v>
       </c>
       <c r="D145" t="n">
         <v>0</v>
       </c>
       <c r="E145" t="n">
-        <v>0.4556677276032285</v>
+        <v>0.6325729579804765</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -3922,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="E146" t="n">
-        <v>0.8570717594710897</v>
+        <v>0.8570717594710898</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3940,16 +3940,16 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-0.006193425526774745</v>
+        <v>-0.006193425526774751</v>
       </c>
       <c r="D147" t="n">
-        <v>0.5619864729076206</v>
+        <v>0.7378467612699779</v>
       </c>
       <c r="E147" t="n">
         <v>0.03333228346491916</v>
       </c>
       <c r="F147" t="n">
-        <v>0.001797762338643773</v>
+        <v>0.07157179673421588</v>
       </c>
     </row>
     <row r="148">
@@ -3964,13 +3964,13 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>0.7545405682512193</v>
+        <v>0.7545405682512194</v>
       </c>
       <c r="D148" t="n">
         <v>0</v>
       </c>
       <c r="E148" t="n">
-        <v>0.8974345293025542</v>
+        <v>0.8974345293025541</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>0.648218207719039</v>
+        <v>0.6482182077190393</v>
       </c>
       <c r="D149" t="n">
         <v>0</v>
@@ -3997,7 +3997,7 @@
         <v>0.6103058781014912</v>
       </c>
       <c r="F149" t="n">
-        <v>0</v>
+        <v>6.686767738481168e-298</v>
       </c>
     </row>
     <row r="150">
@@ -4012,10 +4012,10 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>0.5724544220071908</v>
+        <v>0.5724544220071909</v>
       </c>
       <c r="D150" t="n">
-        <v>0</v>
+        <v>3.657467494590659e-254</v>
       </c>
       <c r="E150" t="n">
         <v>0.6755834327850317</v>
@@ -4036,13 +4036,13 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>0.9560728157110109</v>
+        <v>0.956072815711011</v>
       </c>
       <c r="D151" t="n">
         <v>0</v>
       </c>
       <c r="E151" t="n">
-        <v>0.9879795733556365</v>
+        <v>0.9879795733556361</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4066,7 +4066,7 @@
         <v>0</v>
       </c>
       <c r="E152" t="n">
-        <v>0.7648115466624595</v>
+        <v>0.7648115466624594</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4084,7 +4084,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>0.8954789419953444</v>
+        <v>0.8954789419953446</v>
       </c>
       <c r="D153" t="n">
         <v>0</v>
@@ -4108,13 +4108,13 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>0.7437421256360544</v>
+        <v>0.7437421256360547</v>
       </c>
       <c r="D154" t="n">
         <v>0</v>
       </c>
       <c r="E154" t="n">
-        <v>0.8193256353355839</v>
+        <v>0.8193256353355838</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4156,16 +4156,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>0.5411762296819582</v>
+        <v>0.5554679531016424</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>2.510018256957381e-236</v>
       </c>
       <c r="E156" t="n">
-        <v>0.5208105274306088</v>
+        <v>0.5307412861331078</v>
       </c>
       <c r="F156" t="n">
-        <v>0</v>
+        <v>3.896550603077885e-212</v>
       </c>
     </row>
     <row r="157">
@@ -4180,16 +4180,16 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>0.4211297586207482</v>
+        <v>0.4178108929886101</v>
       </c>
       <c r="D157" t="n">
-        <v>0</v>
+        <v>7.279130922842563e-124</v>
       </c>
       <c r="E157" t="n">
-        <v>0.3693150134761911</v>
+        <v>0.3654927912779786</v>
       </c>
       <c r="F157" t="n">
-        <v>1.597261145149038e-281</v>
+        <v>4.509022961030906e-93</v>
       </c>
     </row>
     <row r="158">
@@ -4204,16 +4204,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>0.3788870825828101</v>
+        <v>0.371196665058563</v>
       </c>
       <c r="D158" t="n">
-        <v>2.182346851553543e-297</v>
+        <v>3.661922663142359e-96</v>
       </c>
       <c r="E158" t="n">
-        <v>0.356930621467112</v>
+        <v>0.3478765895283323</v>
       </c>
       <c r="F158" t="n">
-        <v>8.753997061692866e-262</v>
+        <v>6.44636304991311e-84</v>
       </c>
     </row>
     <row r="159">
@@ -4228,13 +4228,13 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>0.5873636682854525</v>
+        <v>0.6165019686220626</v>
       </c>
       <c r="D159" t="n">
-        <v>0</v>
+        <v>1.232027484628098e-305</v>
       </c>
       <c r="E159" t="n">
-        <v>0.5996507743271579</v>
+        <v>0.683381893463609</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4252,13 +4252,13 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>0.5576555203472524</v>
+        <v>0.809061271942215</v>
       </c>
       <c r="D160" t="n">
         <v>0</v>
       </c>
       <c r="E160" t="n">
-        <v>0.5477607666539643</v>
+        <v>0.7624071708546051</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4276,13 +4276,13 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>0.5379296732524539</v>
+        <v>0.7805743049531599</v>
       </c>
       <c r="D161" t="n">
         <v>0</v>
       </c>
       <c r="E161" t="n">
-        <v>0.5419105841919781</v>
+        <v>0.7569341245985597</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4300,16 +4300,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>0.5670732446468155</v>
+        <v>0.5684727299689658</v>
       </c>
       <c r="D162" t="n">
-        <v>0</v>
+        <v>6.88300222684879e-250</v>
       </c>
       <c r="E162" t="n">
-        <v>0.5102688149832127</v>
+        <v>0.5099218927224485</v>
       </c>
       <c r="F162" t="n">
-        <v>0</v>
+        <v>2.862243632667048e-193</v>
       </c>
     </row>
     <row r="163">
@@ -4324,16 +4324,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>0.01018635663702321</v>
+        <v>0.02136207992481769</v>
       </c>
       <c r="D163" t="n">
-        <v>0.3402005177178452</v>
+        <v>0.248264997446791</v>
       </c>
       <c r="E163" t="n">
-        <v>0.00209276792432931</v>
+        <v>0.02881592477610772</v>
       </c>
       <c r="F163" t="n">
-        <v>0.8446530459048818</v>
+        <v>0.1193319946773843</v>
       </c>
     </row>
     <row r="164">
@@ -4348,16 +4348,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>0.760419829557472</v>
+        <v>0.7890124800257879</v>
       </c>
       <c r="D164" t="n">
         <v>0</v>
       </c>
       <c r="E164" t="n">
-        <v>0.5022567308757648</v>
+        <v>0.5112367995252334</v>
       </c>
       <c r="F164" t="n">
-        <v>0</v>
+        <v>2.011876431627369e-194</v>
       </c>
     </row>
     <row r="165">
@@ -4372,16 +4372,16 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>0.3216738536245097</v>
+        <v>0.3377286666969999</v>
       </c>
       <c r="D165" t="n">
-        <v>3.033455259270989e-210</v>
+        <v>6.651981994021564e-79</v>
       </c>
       <c r="E165" t="n">
-        <v>0.3742853801281313</v>
+        <v>0.3727386080762574</v>
       </c>
       <c r="F165" t="n">
-        <v>1.078262449473593e-289</v>
+        <v>5.217798937917992e-97</v>
       </c>
     </row>
     <row r="166">
@@ -4396,16 +4396,16 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>0.3898379176770721</v>
+        <v>0.4035643370018586</v>
       </c>
       <c r="D166" t="n">
-        <v>3.325232842038179e-316</v>
+        <v>6.396129474769507e-115</v>
       </c>
       <c r="E166" t="n">
-        <v>0.4110417597634477</v>
+        <v>0.4141971159420432</v>
       </c>
       <c r="F166" t="n">
-        <v>0</v>
+        <v>1.486165612633583e-121</v>
       </c>
     </row>
     <row r="167">
@@ -4420,16 +4420,16 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>0.4682599022735286</v>
+        <v>0.4775889959796603</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>1.904024295814503e-166</v>
       </c>
       <c r="E167" t="n">
-        <v>0.5151193076879514</v>
+        <v>0.5309792149274541</v>
       </c>
       <c r="F167" t="n">
-        <v>0</v>
+        <v>2.330146312206435e-212</v>
       </c>
     </row>
     <row r="168">
@@ -4444,16 +4444,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>0.6397064258770415</v>
+        <v>0.6414291219845514</v>
       </c>
       <c r="D168" t="n">
         <v>0</v>
       </c>
       <c r="E168" t="n">
-        <v>0.4996094804981535</v>
+        <v>0.486740055226751</v>
       </c>
       <c r="F168" t="n">
-        <v>0</v>
+        <v>9.514259742322854e-174</v>
       </c>
     </row>
     <row r="169">
@@ -4468,16 +4468,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>0.5926228087235358</v>
+        <v>0.5954241994209174</v>
       </c>
       <c r="D169" t="n">
-        <v>0</v>
+        <v>5.224581382714567e-280</v>
       </c>
       <c r="E169" t="n">
-        <v>0.5057841390057547</v>
+        <v>0.5070053234883386</v>
       </c>
       <c r="F169" t="n">
-        <v>0</v>
+        <v>9.917867204668648e-191</v>
       </c>
     </row>
     <row r="170">
@@ -4492,16 +4492,16 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>0.4087122424828521</v>
+        <v>0.4153143148941014</v>
       </c>
       <c r="D170" t="n">
-        <v>0</v>
+        <v>2.890441153326847e-122</v>
       </c>
       <c r="E170" t="n">
-        <v>0.4582765507040158</v>
+        <v>0.4682918695866836</v>
       </c>
       <c r="F170" t="n">
-        <v>0</v>
+        <v>2.974753368755851e-159</v>
       </c>
     </row>
     <row r="171">
@@ -4516,16 +4516,16 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>0.5411762296819582</v>
+        <v>0.5554679531016424</v>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>2.510018256957381e-236</v>
       </c>
       <c r="E171" t="n">
-        <v>0.5208105274306088</v>
+        <v>0.5307412861331078</v>
       </c>
       <c r="F171" t="n">
-        <v>0</v>
+        <v>3.896550603077885e-212</v>
       </c>
     </row>
     <row r="172">
@@ -4564,13 +4564,13 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>0.6761727267539888</v>
+        <v>0.6594957835569841</v>
       </c>
       <c r="D173" t="n">
         <v>0</v>
       </c>
       <c r="E173" t="n">
-        <v>0.8785070937454584</v>
+        <v>0.8812943880399026</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4588,13 +4588,13 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>0.60700825324538</v>
+        <v>0.5857556869575522</v>
       </c>
       <c r="D174" t="n">
-        <v>0</v>
+        <v>7.069984402404505e-269</v>
       </c>
       <c r="E174" t="n">
-        <v>0.8548466163769821</v>
+        <v>0.8587938329286099</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -4612,16 +4612,16 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>0.710396939507975</v>
+        <v>0.8196774537063102</v>
       </c>
       <c r="D175" t="n">
         <v>0</v>
       </c>
       <c r="E175" t="n">
-        <v>0.3537914807291565</v>
+        <v>0.4834169162227278</v>
       </c>
       <c r="F175" t="n">
-        <v>6.415970146991912e-257</v>
+        <v>4.523830986051027e-171</v>
       </c>
     </row>
     <row r="176">
@@ -4636,16 +4636,16 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>0.3254816895013254</v>
+        <v>0.5729989538403589</v>
       </c>
       <c r="D176" t="n">
-        <v>1.725403259453431e-215</v>
+        <v>9.419392525395384e-255</v>
       </c>
       <c r="E176" t="n">
-        <v>0.2628046872599911</v>
+        <v>0.510548982248339</v>
       </c>
       <c r="F176" t="n">
-        <v>1.843090312896932e-138</v>
+        <v>8.080014580943635e-194</v>
       </c>
     </row>
     <row r="177">
@@ -4660,16 +4660,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>0.2885858549960023</v>
+        <v>0.5082252143783464</v>
       </c>
       <c r="D177" t="n">
-        <v>8.522306802507747e-168</v>
+        <v>8.652775827035847e-192</v>
       </c>
       <c r="E177" t="n">
-        <v>0.2718798949110201</v>
+        <v>0.5110695594022377</v>
       </c>
       <c r="F177" t="n">
-        <v>2.004232315448521e-148</v>
+        <v>2.821909313689259e-194</v>
       </c>
     </row>
     <row r="178">
@@ -4684,16 +4684,16 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>0.3804040237552211</v>
+        <v>0.3563488844225775</v>
       </c>
       <c r="D178" t="n">
-        <v>5.959553720780655e-300</v>
+        <v>3.011554709451239e-88</v>
       </c>
       <c r="E178" t="n">
-        <v>0.3570458973800983</v>
+        <v>0.3398151892953558</v>
       </c>
       <c r="F178" t="n">
-        <v>5.787577252416711e-262</v>
+        <v>6.417107963704902e-80</v>
       </c>
     </row>
     <row r="179">
@@ -4708,16 +4708,16 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>0.03556791456214933</v>
+        <v>0.04904760331398789</v>
       </c>
       <c r="D179" t="n">
-        <v>0.000864528154016306</v>
+        <v>0.007996685747225583</v>
       </c>
       <c r="E179" t="n">
-        <v>0.02258309947248789</v>
+        <v>0.05207928064780149</v>
       </c>
       <c r="F179" t="n">
-        <v>0.0344541599910787</v>
+        <v>0.004857097301179664</v>
       </c>
     </row>
     <row r="180">
@@ -4732,16 +4732,16 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>0.3122521915572819</v>
+        <v>0.3127661477912633</v>
       </c>
       <c r="D180" t="n">
-        <v>1.365740522621185e-197</v>
+        <v>2.379013604190403e-67</v>
       </c>
       <c r="E180" t="n">
-        <v>0.3110540411491127</v>
+        <v>0.2978604677688969</v>
       </c>
       <c r="F180" t="n">
-        <v>5.148879785190342e-196</v>
+        <v>5.814663421907305e-61</v>
       </c>
     </row>
     <row r="181">
@@ -4756,16 +4756,16 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>0.3072852859526205</v>
+        <v>0.3051606447703192</v>
       </c>
       <c r="D181" t="n">
-        <v>4.190682509214775e-191</v>
+        <v>4.81482132939331e-64</v>
       </c>
       <c r="E181" t="n">
-        <v>0.2734766478441396</v>
+        <v>0.2677579467456537</v>
       </c>
       <c r="F181" t="n">
-        <v>3.22464742660719e-150</v>
+        <v>3.566234961241895e-49</v>
       </c>
     </row>
     <row r="182">
@@ -4780,16 +4780,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>0.2790712506792598</v>
+        <v>0.2847902877252663</v>
       </c>
       <c r="D182" t="n">
-        <v>1.343933497167525e-156</v>
+        <v>1.154579806920999e-55</v>
       </c>
       <c r="E182" t="n">
-        <v>0.2632974146446778</v>
+        <v>0.2592221647068217</v>
       </c>
       <c r="F182" t="n">
-        <v>5.42694288762349e-139</v>
+        <v>4.287620295322336e-46</v>
       </c>
     </row>
     <row r="183">
@@ -4804,16 +4804,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>0.4075747514081423</v>
+        <v>0.4097093086883555</v>
       </c>
       <c r="D183" t="n">
-        <v>0</v>
+        <v>1.003364342699127e-118</v>
       </c>
       <c r="E183" t="n">
-        <v>0.3653004039185452</v>
+        <v>0.3678999806840161</v>
       </c>
       <c r="F183" t="n">
-        <v>4.991471081811902e-275</v>
+        <v>2.277707968055732e-94</v>
       </c>
     </row>
     <row r="184">
@@ -4828,16 +4828,16 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>0.3363603250452208</v>
+        <v>0.3207630264187031</v>
       </c>
       <c r="D184" t="n">
-        <v>6.756398178713562e-231</v>
+        <v>6.216881795166131e-71</v>
       </c>
       <c r="E184" t="n">
-        <v>0.3303190646088016</v>
+        <v>0.3069814252586165</v>
       </c>
       <c r="F184" t="n">
-        <v>2.907871889481965e-222</v>
+        <v>7.942911745145299e-65</v>
       </c>
     </row>
     <row r="185">
@@ -4852,16 +4852,16 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>0.3937841663624979</v>
+        <v>0.3803380055735273</v>
       </c>
       <c r="D185" t="n">
-        <v>3.952525166729972e-323</v>
+        <v>3.013079602062415e-101</v>
       </c>
       <c r="E185" t="n">
-        <v>0.3527963077087693</v>
+        <v>0.3402221413844022</v>
       </c>
       <c r="F185" t="n">
-        <v>2.178008683113858e-255</v>
+        <v>4.058274053945986e-80</v>
       </c>
     </row>
     <row r="186">
@@ -4876,16 +4876,16 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>0.3503533015298208</v>
+        <v>0.3575538183550458</v>
       </c>
       <c r="D186" t="n">
-        <v>1.181761123760613e-251</v>
+        <v>7.112860809889674e-89</v>
       </c>
       <c r="E186" t="n">
-        <v>0.320934890156163</v>
+        <v>0.3191854015970586</v>
       </c>
       <c r="F186" t="n">
-        <v>3.097555130847909e-209</v>
+        <v>3.229370326874344e-70</v>
       </c>
     </row>
     <row r="187">
@@ -4900,16 +4900,16 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>0.4211297586207482</v>
+        <v>0.4178108929886101</v>
       </c>
       <c r="D187" t="n">
-        <v>0</v>
+        <v>7.279130922842563e-124</v>
       </c>
       <c r="E187" t="n">
-        <v>0.3693150134761911</v>
+        <v>0.3654927912779787</v>
       </c>
       <c r="F187" t="n">
-        <v>1.597261145149038e-281</v>
+        <v>4.509022961030649e-93</v>
       </c>
     </row>
     <row r="188">
@@ -4924,13 +4924,13 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>0.6761727267539888</v>
+        <v>0.6594957835569841</v>
       </c>
       <c r="D188" t="n">
         <v>0</v>
       </c>
       <c r="E188" t="n">
-        <v>0.8785070937454583</v>
+        <v>0.8812943880399026</v>
       </c>
       <c r="F188" t="n">
         <v>0</v>
@@ -4948,7 +4948,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D189" t="n">
         <v>0</v>
@@ -4972,13 +4972,13 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>0.9609733185846652</v>
+        <v>0.9654277884779845</v>
       </c>
       <c r="D190" t="n">
         <v>0</v>
       </c>
       <c r="E190" t="n">
-        <v>0.9819700313368082</v>
+        <v>0.9852574468409722</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -4996,16 +4996,16 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>0.2714828690285614</v>
+        <v>0.3313604009513878</v>
       </c>
       <c r="D191" t="n">
-        <v>5.571854781952344e-148</v>
+        <v>7.489763442248213e-76</v>
       </c>
       <c r="E191" t="n">
-        <v>0.1894042201512334</v>
+        <v>0.3077832201017826</v>
       </c>
       <c r="F191" t="n">
-        <v>1.265793538845598e-71</v>
+        <v>3.577523718702434e-65</v>
       </c>
     </row>
     <row r="192">
@@ -5020,16 +5020,16 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>0.2101518712017543</v>
+        <v>0.4411146101364154</v>
       </c>
       <c r="D192" t="n">
-        <v>4.148064780803994e-88</v>
+        <v>1.853740652988266e-139</v>
       </c>
       <c r="E192" t="n">
-        <v>0.1592927497948927</v>
+        <v>0.3843570326953448</v>
       </c>
       <c r="F192" t="n">
-        <v>6.272114226109191e-51</v>
+        <v>1.553486734833515e-103</v>
       </c>
     </row>
     <row r="193">
@@ -5044,16 +5044,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>0.204187365146615</v>
+        <v>0.4432493998554754</v>
       </c>
       <c r="D193" t="n">
-        <v>3.516044650648705e-83</v>
+        <v>5.989911573938559e-141</v>
       </c>
       <c r="E193" t="n">
-        <v>0.1711140866145746</v>
+        <v>0.3839291352356591</v>
       </c>
       <c r="F193" t="n">
-        <v>1.324281859025998e-58</v>
+        <v>2.731534893949845e-103</v>
       </c>
     </row>
     <row r="194">
@@ -5068,16 +5068,16 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>0.3408724811364616</v>
+        <v>0.313299611122669</v>
       </c>
       <c r="D194" t="n">
-        <v>1.791022551291699e-237</v>
+        <v>1.382952935969628e-67</v>
       </c>
       <c r="E194" t="n">
-        <v>0.3482939178534328</v>
+        <v>0.3234651887045832</v>
       </c>
       <c r="F194" t="n">
-        <v>1.566161604565199e-248</v>
+        <v>3.613664906637146e-72</v>
       </c>
     </row>
     <row r="195">
@@ -5092,16 +5092,16 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>0.03933753877822468</v>
+        <v>0.05328252544415385</v>
       </c>
       <c r="D195" t="n">
-        <v>0.0002290767573875307</v>
+        <v>0.003957588779356236</v>
       </c>
       <c r="E195" t="n">
-        <v>0.03107442286039943</v>
+        <v>0.05892823236329751</v>
       </c>
       <c r="F195" t="n">
-        <v>0.003612111865458417</v>
+        <v>0.001435834573158047</v>
       </c>
     </row>
     <row r="196">
@@ -5116,16 +5116,16 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>0.2499247158382008</v>
+        <v>0.2476585478192828</v>
       </c>
       <c r="D196" t="n">
-        <v>5.552230875591728e-125</v>
+        <v>4.216682433567577e-42</v>
       </c>
       <c r="E196" t="n">
-        <v>0.3000647671265144</v>
+        <v>0.2806919673166814</v>
       </c>
       <c r="F196" t="n">
-        <v>6.751879545148911e-182</v>
+        <v>4.638489294353596e-54</v>
       </c>
     </row>
     <row r="197">
@@ -5140,16 +5140,16 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>0.2709268150383519</v>
+        <v>0.2669209206728209</v>
       </c>
       <c r="D197" t="n">
-        <v>2.326242065173933e-147</v>
+        <v>7.232289635408424e-49</v>
       </c>
       <c r="E197" t="n">
-        <v>0.2489887219065404</v>
+        <v>0.2417839643056925</v>
       </c>
       <c r="F197" t="n">
-        <v>4.944103699853044e-124</v>
+        <v>3.760334409000857e-40</v>
       </c>
     </row>
     <row r="198">
@@ -5164,16 +5164,16 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>0.2768588934974741</v>
+        <v>0.2746780170093809</v>
       </c>
       <c r="D198" t="n">
-        <v>4.669965564166831e-154</v>
+        <v>9.35896526804541e-52</v>
       </c>
       <c r="E198" t="n">
-        <v>0.2607033179582323</v>
+        <v>0.2515153802441717</v>
       </c>
       <c r="F198" t="n">
-        <v>3.291013377008339e-136</v>
+        <v>2.070398809269987e-43</v>
       </c>
     </row>
     <row r="199">
@@ -5188,16 +5188,16 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>0.4024488583609284</v>
+        <v>0.3965830112864861</v>
       </c>
       <c r="D199" t="n">
-        <v>0</v>
+        <v>1.076249882176215e-110</v>
       </c>
       <c r="E199" t="n">
-        <v>0.3632729494628876</v>
+        <v>0.359509089290786</v>
       </c>
       <c r="F199" t="n">
-        <v>8.770362586649324e-272</v>
+        <v>6.74847701327128e-90</v>
       </c>
     </row>
     <row r="200">
@@ -5212,16 +5212,16 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>0.2977541246723888</v>
+        <v>0.2782355284792996</v>
       </c>
       <c r="D200" t="n">
-        <v>5.254068579704514e-179</v>
+        <v>4.119046442912065e-53</v>
       </c>
       <c r="E200" t="n">
-        <v>0.3270831565247423</v>
+        <v>0.2962339110355097</v>
       </c>
       <c r="F200" t="n">
-        <v>1.019080151527884e-217</v>
+        <v>2.748727289608711e-60</v>
       </c>
     </row>
     <row r="201">
@@ -5236,16 +5236,16 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>0.3565116123064391</v>
+        <v>0.3386504491435319</v>
       </c>
       <c r="D201" t="n">
-        <v>3.933607204706318e-261</v>
+        <v>2.372692861003124e-79</v>
       </c>
       <c r="E201" t="n">
-        <v>0.3453077374009511</v>
+        <v>0.3267396849040175</v>
       </c>
       <c r="F201" t="n">
-        <v>4.793936916330531e-244</v>
+        <v>1.105450914403047e-73</v>
       </c>
     </row>
     <row r="202">
@@ -5260,16 +5260,16 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>0.3691561116430949</v>
+        <v>0.3623410734346686</v>
       </c>
       <c r="D202" t="n">
-        <v>2.898801059733938e-281</v>
+        <v>2.162462502322655e-91</v>
       </c>
       <c r="E202" t="n">
-        <v>0.3282896131279908</v>
+        <v>0.3190909052808025</v>
       </c>
       <c r="F202" t="n">
-        <v>2.090738171857424e-219</v>
+        <v>3.563204494876834e-70</v>
       </c>
     </row>
     <row r="203">
@@ -5284,16 +5284,16 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>0.3788870825828101</v>
+        <v>0.371196665058563</v>
       </c>
       <c r="D203" t="n">
-        <v>2.182346851553543e-297</v>
+        <v>3.661922663142359e-96</v>
       </c>
       <c r="E203" t="n">
-        <v>0.356930621467112</v>
+        <v>0.3478765895283323</v>
       </c>
       <c r="F203" t="n">
-        <v>8.753997061692866e-262</v>
+        <v>6.446363049913846e-84</v>
       </c>
     </row>
     <row r="204">
@@ -5308,13 +5308,13 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>0.60700825324538</v>
+        <v>0.5857556869575522</v>
       </c>
       <c r="D204" t="n">
-        <v>0</v>
+        <v>7.069984402404505e-269</v>
       </c>
       <c r="E204" t="n">
-        <v>0.8548466163769821</v>
+        <v>0.8587938329286099</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5332,13 +5332,13 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>0.9609733185846652</v>
+        <v>0.9654277884779845</v>
       </c>
       <c r="D205" t="n">
         <v>0</v>
       </c>
       <c r="E205" t="n">
-        <v>0.981970031336808</v>
+        <v>0.9852574468409722</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -5356,7 +5356,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>0.9999999999999999</v>
+        <v>0.9999999999999998</v>
       </c>
       <c r="D206" t="n">
         <v>0</v>
@@ -5380,16 +5380,16 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>0.2163691886146475</v>
+        <v>0.2668399006729145</v>
       </c>
       <c r="D207" t="n">
-        <v>2.071608747449963e-93</v>
+        <v>7.743545898198044e-49</v>
       </c>
       <c r="E207" t="n">
-        <v>0.2004616052907031</v>
+        <v>0.3101706079201246</v>
       </c>
       <c r="F207" t="n">
-        <v>3.520734389034639e-80</v>
+        <v>3.2788776090191e-66</v>
       </c>
     </row>
     <row r="208">
@@ -5404,16 +5404,16 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>0.1961559599253933</v>
+        <v>0.4001589195135647</v>
       </c>
       <c r="D208" t="n">
-        <v>8.7116152972719e-77</v>
+        <v>7.585761109705164e-113</v>
       </c>
       <c r="E208" t="n">
-        <v>0.1753738854905618</v>
+        <v>0.3856543206679376</v>
       </c>
       <c r="F208" t="n">
-        <v>1.638995491345456e-61</v>
+        <v>2.792421354194199e-104</v>
       </c>
     </row>
     <row r="209">
@@ -5428,16 +5428,16 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>0.2173614340535197</v>
+        <v>0.4379132393492713</v>
       </c>
       <c r="D209" t="n">
-        <v>2.848348287956501e-94</v>
+        <v>3.044453191067679e-137</v>
       </c>
       <c r="E209" t="n">
-        <v>0.1937083760645016</v>
+        <v>0.3918497771306699</v>
       </c>
       <c r="F209" t="n">
-        <v>6.821262484235549e-75</v>
+        <v>6.913949627645607e-108</v>
       </c>
     </row>
     <row r="210">
@@ -5452,16 +5452,16 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>0.5962543989652713</v>
+        <v>0.628577020052814</v>
       </c>
       <c r="D210" t="n">
-        <v>0</v>
+        <v>3.231189323801752e-321</v>
       </c>
       <c r="E210" t="n">
-        <v>0.548409526852994</v>
+        <v>0.6173697683708295</v>
       </c>
       <c r="F210" t="n">
-        <v>0</v>
+        <v>9.851530546739947e-307</v>
       </c>
     </row>
     <row r="211">
@@ -5476,16 +5476,16 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>-0.006270023464504971</v>
+        <v>-0.02123838118700429</v>
       </c>
       <c r="D211" t="n">
-        <v>0.5571597220133419</v>
+        <v>0.2510153606089161</v>
       </c>
       <c r="E211" t="n">
-        <v>-0.02733332888341927</v>
+        <v>-0.04200584302493246</v>
       </c>
       <c r="F211" t="n">
-        <v>0.01047666063015807</v>
+        <v>0.02314289370526416</v>
       </c>
     </row>
     <row r="212">
@@ -5500,13 +5500,13 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>0.8162022175137893</v>
+        <v>0.8874025204297278</v>
       </c>
       <c r="D212" t="n">
         <v>0</v>
       </c>
       <c r="E212" t="n">
-        <v>0.6666910856063926</v>
+        <v>0.7725366917449678</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -5524,16 +5524,16 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>0.3301780681499282</v>
+        <v>0.3290533978379733</v>
       </c>
       <c r="D213" t="n">
-        <v>4.599953061782032e-222</v>
+        <v>9.165099730651372e-75</v>
       </c>
       <c r="E213" t="n">
-        <v>0.373118984834427</v>
+        <v>0.4105381974221958</v>
       </c>
       <c r="F213" t="n">
-        <v>9.185084275076665e-288</v>
+        <v>3.034812928967799e-119</v>
       </c>
     </row>
     <row r="214">
@@ -5548,16 +5548,16 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>0.3703949996998294</v>
+        <v>0.3965453382286718</v>
       </c>
       <c r="D214" t="n">
-        <v>2.755846669117891e-283</v>
+        <v>1.133556306195914e-110</v>
       </c>
       <c r="E214" t="n">
-        <v>0.4374669261133945</v>
+        <v>0.5018445951260092</v>
       </c>
       <c r="F214" t="n">
-        <v>0</v>
+        <v>2.693349665732633e-186</v>
       </c>
     </row>
     <row r="215">
@@ -5572,13 +5572,13 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>0.5019743068575309</v>
+        <v>0.5194246389965358</v>
       </c>
       <c r="D215" t="n">
-        <v>0</v>
+        <v>1.019307778738693e-201</v>
       </c>
       <c r="E215" t="n">
-        <v>0.5916864228596775</v>
+        <v>0.6748576249077125</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5596,16 +5596,16 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>0.6683247652977408</v>
+        <v>0.6935080803768686</v>
       </c>
       <c r="D216" t="n">
         <v>0</v>
       </c>
       <c r="E216" t="n">
-        <v>0.5188769338767233</v>
+        <v>0.5635413535925445</v>
       </c>
       <c r="F216" t="n">
-        <v>0</v>
+        <v>1.125979450288559e-244</v>
       </c>
     </row>
     <row r="217">
@@ -5620,13 +5620,13 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>0.630015091868017</v>
+        <v>0.6679093753194176</v>
       </c>
       <c r="D217" t="n">
         <v>0</v>
       </c>
       <c r="E217" t="n">
-        <v>0.5796138633438633</v>
+        <v>0.6590162017447879</v>
       </c>
       <c r="F217" t="n">
         <v>0</v>
@@ -5644,16 +5644,16 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>0.4233697610687855</v>
+        <v>0.4357215233182617</v>
       </c>
       <c r="D218" t="n">
-        <v>0</v>
+        <v>9.695603760244763e-136</v>
       </c>
       <c r="E218" t="n">
-        <v>0.5234867060019465</v>
+        <v>0.5955793106741324</v>
       </c>
       <c r="F218" t="n">
-        <v>0</v>
+        <v>3.438548842950038e-280</v>
       </c>
     </row>
     <row r="219">
@@ -5668,13 +5668,13 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>0.5873636682854525</v>
+        <v>0.6165019686220627</v>
       </c>
       <c r="D219" t="n">
-        <v>0</v>
+        <v>1.232027484627774e-305</v>
       </c>
       <c r="E219" t="n">
-        <v>0.5996507743271579</v>
+        <v>0.683381893463609</v>
       </c>
       <c r="F219" t="n">
         <v>0</v>
@@ -5692,16 +5692,16 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>0.710396939507975</v>
+        <v>0.8196774537063102</v>
       </c>
       <c r="D220" t="n">
         <v>0</v>
       </c>
       <c r="E220" t="n">
-        <v>0.3537914807291565</v>
+        <v>0.4834169162227278</v>
       </c>
       <c r="F220" t="n">
-        <v>6.415970146991912e-257</v>
+        <v>4.523830986051027e-171</v>
       </c>
     </row>
     <row r="221">
@@ -5716,16 +5716,16 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>0.2714828690285614</v>
+        <v>0.3313604009513878</v>
       </c>
       <c r="D221" t="n">
-        <v>5.571854781952344e-148</v>
+        <v>7.489763442248213e-76</v>
       </c>
       <c r="E221" t="n">
-        <v>0.1894042201512334</v>
+        <v>0.3077832201017826</v>
       </c>
       <c r="F221" t="n">
-        <v>1.265793538845598e-71</v>
+        <v>3.577523718702434e-65</v>
       </c>
     </row>
     <row r="222">
@@ -5740,16 +5740,16 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>0.2163691886146475</v>
+        <v>0.2668399006729145</v>
       </c>
       <c r="D222" t="n">
-        <v>2.071608747449963e-93</v>
+        <v>7.743545898198044e-49</v>
       </c>
       <c r="E222" t="n">
-        <v>0.2004616052907031</v>
+        <v>0.3101706079201246</v>
       </c>
       <c r="F222" t="n">
-        <v>3.520734389034639e-80</v>
+        <v>3.2788776090191e-66</v>
       </c>
     </row>
     <row r="223">
@@ -5788,13 +5788,13 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>0.7286702979134105</v>
+        <v>0.728298171217165</v>
       </c>
       <c r="D224" t="n">
         <v>0</v>
       </c>
       <c r="E224" t="n">
-        <v>0.8905803499178149</v>
+        <v>0.9015543669352931</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -5812,13 +5812,13 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>0.6730239502066849</v>
+        <v>0.6465618721814568</v>
       </c>
       <c r="D225" t="n">
         <v>0</v>
       </c>
       <c r="E225" t="n">
-        <v>0.8832931717617204</v>
+        <v>0.8992352324220696</v>
       </c>
       <c r="F225" t="n">
         <v>0</v>
@@ -5836,13 +5836,13 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>0.4661975474024565</v>
+        <v>0.6727347821300382</v>
       </c>
       <c r="D226" t="n">
         <v>0</v>
       </c>
       <c r="E226" t="n">
-        <v>0.4774599582613798</v>
+        <v>0.6564237649531522</v>
       </c>
       <c r="F226" t="n">
         <v>0</v>
@@ -5860,16 +5860,16 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>0.02697172857219367</v>
+        <v>-0.0001618543403799661</v>
       </c>
       <c r="D227" t="n">
-        <v>0.01154314507902686</v>
+        <v>0.9930210918079525</v>
       </c>
       <c r="E227" t="n">
-        <v>0.03049910076868118</v>
+        <v>0.03829958830482363</v>
       </c>
       <c r="F227" t="n">
-        <v>0.004286333051198726</v>
+        <v>0.03840249404038574</v>
       </c>
     </row>
     <row r="228">
@@ -5884,13 +5884,13 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>0.3984232096795319</v>
+        <v>0.6017818671719291</v>
       </c>
       <c r="D228" t="n">
-        <v>0</v>
+        <v>1.54678419033053e-287</v>
       </c>
       <c r="E228" t="n">
-        <v>0.4831313822728238</v>
+        <v>0.68003028541919</v>
       </c>
       <c r="F228" t="n">
         <v>0</v>
@@ -5908,16 +5908,16 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.3715616261543613</v>
+        <v>0.4985624511795598</v>
       </c>
       <c r="D229" t="n">
-        <v>3.373432845809345e-285</v>
+        <v>1.624781270499516e-183</v>
       </c>
       <c r="E229" t="n">
-        <v>0.3532439313403115</v>
+        <v>0.4682609954027203</v>
       </c>
       <c r="F229" t="n">
-        <v>4.468890820878274e-256</v>
+        <v>3.140302652040833e-159</v>
       </c>
     </row>
     <row r="230">
@@ -5932,16 +5932,16 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>0.3089852309067529</v>
+        <v>0.4561969243634081</v>
       </c>
       <c r="D230" t="n">
-        <v>2.607758478347649e-193</v>
+        <v>3.198415177047571e-150</v>
       </c>
       <c r="E230" t="n">
-        <v>0.3582279529335333</v>
+        <v>0.501312573825911</v>
       </c>
       <c r="F230" t="n">
-        <v>8.230089132646972e-264</v>
+        <v>7.639505610511546e-186</v>
       </c>
     </row>
     <row r="231">
@@ -5956,13 +5956,13 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>0.529936387048587</v>
+        <v>0.7561706466631242</v>
       </c>
       <c r="D231" t="n">
         <v>0</v>
       </c>
       <c r="E231" t="n">
-        <v>0.5411708015366777</v>
+        <v>0.7551411147977549</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -5980,16 +5980,16 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>0.4201886578392034</v>
+        <v>0.5685183567514942</v>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>6.153545989357209e-250</v>
       </c>
       <c r="E232" t="n">
-        <v>0.4372618026972731</v>
+        <v>0.5846701978281482</v>
       </c>
       <c r="F232" t="n">
-        <v>0</v>
+        <v>1.190708871335987e-267</v>
       </c>
     </row>
     <row r="233">
@@ -6004,13 +6004,13 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>0.5025739628471854</v>
+        <v>0.7336547611954214</v>
       </c>
       <c r="D233" t="n">
         <v>0</v>
       </c>
       <c r="E233" t="n">
-        <v>0.5063145748881588</v>
+        <v>0.7036176710225318</v>
       </c>
       <c r="F233" t="n">
         <v>0</v>
@@ -6028,16 +6028,16 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>0.4227601785774302</v>
+        <v>0.5972439902745043</v>
       </c>
       <c r="D234" t="n">
-        <v>0</v>
+        <v>3.804793221767193e-282</v>
       </c>
       <c r="E234" t="n">
-        <v>0.4525712442293983</v>
+        <v>0.6305744038468284</v>
       </c>
       <c r="F234" t="n">
-        <v>0</v>
+        <v>9.881312916824931e-324</v>
       </c>
     </row>
     <row r="235">
@@ -6052,13 +6052,13 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>0.5576555203472523</v>
+        <v>0.8090612719422149</v>
       </c>
       <c r="D235" t="n">
         <v>0</v>
       </c>
       <c r="E235" t="n">
-        <v>0.5477607666539643</v>
+        <v>0.7624071708546052</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -6076,16 +6076,16 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>0.3254816895013254</v>
+        <v>0.5729989538403589</v>
       </c>
       <c r="D236" t="n">
-        <v>1.725403259453431e-215</v>
+        <v>9.419392525395384e-255</v>
       </c>
       <c r="E236" t="n">
-        <v>0.2628046872599911</v>
+        <v>0.510548982248339</v>
       </c>
       <c r="F236" t="n">
-        <v>1.843090312896932e-138</v>
+        <v>8.080014580943635e-194</v>
       </c>
     </row>
     <row r="237">
@@ -6100,16 +6100,16 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0.2101518712017543</v>
+        <v>0.4411146101364154</v>
       </c>
       <c r="D237" t="n">
-        <v>4.148064780803994e-88</v>
+        <v>1.853740652988266e-139</v>
       </c>
       <c r="E237" t="n">
-        <v>0.1592927497948926</v>
+        <v>0.3843570326953448</v>
       </c>
       <c r="F237" t="n">
-        <v>6.272114226109639e-51</v>
+        <v>1.553486734833515e-103</v>
       </c>
     </row>
     <row r="238">
@@ -6124,16 +6124,16 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>0.1961559599253933</v>
+        <v>0.4001589195135647</v>
       </c>
       <c r="D238" t="n">
-        <v>8.7116152972719e-77</v>
+        <v>7.585761109705164e-113</v>
       </c>
       <c r="E238" t="n">
-        <v>0.1753738854905618</v>
+        <v>0.3856543206679376</v>
       </c>
       <c r="F238" t="n">
-        <v>1.638995491345456e-61</v>
+        <v>2.792421354193881e-104</v>
       </c>
     </row>
     <row r="239">
@@ -6148,13 +6148,13 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>0.7286702979134105</v>
+        <v>0.728298171217165</v>
       </c>
       <c r="D239" t="n">
         <v>0</v>
       </c>
       <c r="E239" t="n">
-        <v>0.890580349917815</v>
+        <v>0.9015543669352932</v>
       </c>
       <c r="F239" t="n">
         <v>0</v>
@@ -6196,13 +6196,13 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0.9688011573915183</v>
+        <v>0.9581370003729293</v>
       </c>
       <c r="D241" t="n">
         <v>0</v>
       </c>
       <c r="E241" t="n">
-        <v>0.9916811718851848</v>
+        <v>0.9939141404661613</v>
       </c>
       <c r="F241" t="n">
         <v>0</v>
@@ -6220,13 +6220,13 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0.4406584047088115</v>
+        <v>0.6291109304196082</v>
       </c>
       <c r="D242" t="n">
-        <v>0</v>
+        <v>6.422853395936205e-322</v>
       </c>
       <c r="E242" t="n">
-        <v>0.4715663975722654</v>
+        <v>0.6489019349583953</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -6244,16 +6244,16 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0.02701923365697489</v>
+        <v>0.001022159890245563</v>
       </c>
       <c r="D243" t="n">
-        <v>0.01139774940279815</v>
+        <v>0.9559478815990498</v>
       </c>
       <c r="E243" t="n">
-        <v>0.03120036263957241</v>
+        <v>0.0367581525922807</v>
       </c>
       <c r="F243" t="n">
-        <v>0.003478044224510393</v>
+        <v>0.04690657714764744</v>
       </c>
     </row>
     <row r="244">
@@ -6268,13 +6268,13 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0.3570432489558609</v>
+        <v>0.5326142466146806</v>
       </c>
       <c r="D244" t="n">
-        <v>5.842872470064653e-262</v>
+        <v>6.730756418763045e-214</v>
       </c>
       <c r="E244" t="n">
-        <v>0.4799749441437264</v>
+        <v>0.6784089636963448</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -6292,16 +6292,16 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>0.3698856612386199</v>
+        <v>0.4991921632127196</v>
       </c>
       <c r="D245" t="n">
-        <v>1.873329941423436e-282</v>
+        <v>4.782771346255567e-184</v>
       </c>
       <c r="E245" t="n">
-        <v>0.3471667045967565</v>
+        <v>0.4635132422849853</v>
       </c>
       <c r="F245" t="n">
-        <v>7.832752125756156e-247</v>
+        <v>1.216968915903044e-155</v>
       </c>
     </row>
     <row r="246">
@@ -6316,16 +6316,16 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0.3302646504115752</v>
+        <v>0.4874773034984594</v>
       </c>
       <c r="D246" t="n">
-        <v>3.471009545346545e-222</v>
+        <v>2.401189319370942e-174</v>
       </c>
       <c r="E246" t="n">
-        <v>0.3602639731468211</v>
+        <v>0.5044367858557851</v>
       </c>
       <c r="F246" t="n">
-        <v>5.192471947474459e-267</v>
+        <v>1.631999756783036e-188</v>
       </c>
     </row>
     <row r="247">
@@ -6340,13 +6340,13 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0.5523042907844735</v>
+        <v>0.7953303508166576</v>
       </c>
       <c r="D247" t="n">
         <v>0</v>
       </c>
       <c r="E247" t="n">
-        <v>0.5445199998267021</v>
+        <v>0.7603448776971422</v>
       </c>
       <c r="F247" t="n">
         <v>0</v>
@@ -6364,16 +6364,16 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0.3946052730366</v>
+        <v>0.5261332267278964</v>
       </c>
       <c r="D248" t="n">
-        <v>0</v>
+        <v>7.592567275135141e-208</v>
       </c>
       <c r="E248" t="n">
-        <v>0.4353205574189013</v>
+        <v>0.5820603351510775</v>
       </c>
       <c r="F248" t="n">
-        <v>0</v>
+        <v>1.012817295614129e-264</v>
       </c>
     </row>
     <row r="249">
@@ -6388,13 +6388,13 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0.4780327375826023</v>
+        <v>0.6937593939631953</v>
       </c>
       <c r="D249" t="n">
         <v>0</v>
       </c>
       <c r="E249" t="n">
-        <v>0.4998976758143783</v>
+        <v>0.6956324365644663</v>
       </c>
       <c r="F249" t="n">
         <v>0</v>
@@ -6412,13 +6412,13 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0.45402368917089</v>
+        <v>0.6490046574017936</v>
       </c>
       <c r="D250" t="n">
         <v>0</v>
       </c>
       <c r="E250" t="n">
-        <v>0.4556677276032284</v>
+        <v>0.6325729579804766</v>
       </c>
       <c r="F250" t="n">
         <v>0</v>
@@ -6436,13 +6436,13 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>0.5379296732524539</v>
+        <v>0.7805743049531599</v>
       </c>
       <c r="D251" t="n">
         <v>0</v>
       </c>
       <c r="E251" t="n">
-        <v>0.5419105841919781</v>
+        <v>0.7569341245985597</v>
       </c>
       <c r="F251" t="n">
         <v>0</v>
@@ -6460,16 +6460,16 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0.2885858549960023</v>
+        <v>0.5082252143783464</v>
       </c>
       <c r="D252" t="n">
-        <v>8.522306802507747e-168</v>
+        <v>8.652775827035847e-192</v>
       </c>
       <c r="E252" t="n">
-        <v>0.2718798949110201</v>
+        <v>0.5110695594022377</v>
       </c>
       <c r="F252" t="n">
-        <v>2.004232315448521e-148</v>
+        <v>2.821909313689259e-194</v>
       </c>
     </row>
     <row r="253">
@@ -6484,16 +6484,16 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>0.204187365146615</v>
+        <v>0.4432493998554754</v>
       </c>
       <c r="D253" t="n">
-        <v>3.516044650648705e-83</v>
+        <v>5.989911573938559e-141</v>
       </c>
       <c r="E253" t="n">
-        <v>0.1711140866145746</v>
+        <v>0.3839291352356591</v>
       </c>
       <c r="F253" t="n">
-        <v>1.324281859025998e-58</v>
+        <v>2.731534893949845e-103</v>
       </c>
     </row>
     <row r="254">
@@ -6508,16 +6508,16 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>0.2173614340535197</v>
+        <v>0.4379132393492713</v>
       </c>
       <c r="D254" t="n">
-        <v>2.848348287956501e-94</v>
+        <v>3.044453191067679e-137</v>
       </c>
       <c r="E254" t="n">
-        <v>0.1937083760645016</v>
+        <v>0.3918497771306699</v>
       </c>
       <c r="F254" t="n">
-        <v>6.821262484236134e-75</v>
+        <v>6.913949627645212e-108</v>
       </c>
     </row>
     <row r="255">
@@ -6532,13 +6532,13 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>0.6730239502066849</v>
+        <v>0.6465618721814568</v>
       </c>
       <c r="D255" t="n">
         <v>0</v>
       </c>
       <c r="E255" t="n">
-        <v>0.8832931717617203</v>
+        <v>0.8992352324220696</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6556,13 +6556,13 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>0.9688011573915183</v>
+        <v>0.9581370003729293</v>
       </c>
       <c r="D256" t="n">
         <v>0</v>
       </c>
       <c r="E256" t="n">
-        <v>0.9916811718851848</v>
+        <v>0.9939141404661613</v>
       </c>
       <c r="F256" t="n">
         <v>0</v>

</xml_diff>